<commit_message>
Correções no leitor de dados das ações, que não estava tratando bem casos de duplicatas de ticker, ou falta de dados de tickers. Todas as funções foram revisadas para tratar esses casos, gerando novas bases de dados corrigidas
</commit_message>
<xml_diff>
--- a/Bases/Lista de ações Tratada.xlsx
+++ b/Bases/Lista de ações Tratada.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D250"/>
+  <dimension ref="A1:D249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Volume no último dia útil (lido em 15/03/2025)</t>
+          <t>Volume no último dia útil (lido em 16/03/2025)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>42086800</v>
+        <v>42077200</v>
       </c>
       <c r="D7" t="n">
         <v>122790780928</v>
@@ -732,7 +732,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>26742900</v>
+        <v>26742800</v>
       </c>
       <c r="D17" t="n">
         <v>13552640000</v>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>22864500</v>
+        <v>22864700</v>
       </c>
       <c r="D20" t="n">
         <v>159137906688</v>
@@ -2352,7 +2352,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2439300</v>
+        <v>2439400</v>
       </c>
       <c r="D107" t="n">
         <v>4706683392</v>
@@ -4647,288 +4647,270 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>IGTI3</t>
+          <t>TECN3</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Iguatemi</t>
+          <t>Technos</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>62100</v>
+        <v>52700</v>
       </c>
       <c r="D235" t="n">
-        <v>5093064192</v>
+        <v>333557216</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>TECN3</t>
+          <t>ALPK3</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Technos</t>
+          <t>Estapar</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>52700</v>
+        <v>49600</v>
       </c>
       <c r="D236" t="n">
-        <v>333557216</v>
+        <v>625248768</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>ALPK3</t>
+          <t>CSUD3</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Estapar</t>
+          <t>CSU Cardsystem</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>49600</v>
+        <v>47600</v>
       </c>
       <c r="D237" t="n">
-        <v>625248768</v>
+        <v>677006720</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>CSUD3</t>
+          <t>DMVF3</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>CSU Cardsystem</t>
+          <t>D1000 Varejo Farma</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>47600</v>
+        <v>47300</v>
       </c>
       <c r="D238" t="n">
-        <v>677006720</v>
+        <v>303616800</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>DMVF3</t>
+          <t>LOGN3</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>D1000 Varejo Farma</t>
+          <t>Log-In</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>47300</v>
+        <v>41100</v>
       </c>
       <c r="D239" t="n">
-        <v>303616800</v>
+        <v>2280891904</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>LOGN3</t>
+          <t>TCSA3</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Log-In</t>
+          <t>Tecnisa</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>41100</v>
+        <v>39100</v>
       </c>
       <c r="D240" t="n">
-        <v>2280891904</v>
+        <v>106011656</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>TCSA3</t>
+          <t>GOAU3</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Tecnisa</t>
+          <t>Metalúrgica Gerdau</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>39100</v>
+        <v>38900</v>
       </c>
       <c r="D241" t="n">
-        <v>106011656</v>
+        <v>9424949248</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>GOAU3</t>
+          <t>RSID3</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Metalúrgica Gerdau</t>
+          <t>Rossi Residencial</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>38900</v>
+        <v>38700</v>
       </c>
       <c r="D242" t="n">
-        <v>9424949248</v>
+        <v>57684308</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>RSID3</t>
+          <t>BIOM3</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Rossi Residencial</t>
+          <t>Biomm</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>38700</v>
+        <v>38600</v>
       </c>
       <c r="D243" t="n">
-        <v>57684308</v>
+        <v>1291241472</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>BIOM3</t>
+          <t>LVTC3</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Biomm</t>
+          <t>WDC Networks</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>38600</v>
+        <v>26100</v>
       </c>
       <c r="D244" t="n">
-        <v>1291241472</v>
+        <v>155480672</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>LVTC3</t>
+          <t>ALPA3</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>WDC Networks</t>
+          <t>Alpargatas</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>26100</v>
+        <v>25500</v>
       </c>
       <c r="D245" t="n">
-        <v>155480672</v>
+        <v>4706682368</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>ALPA3</t>
+          <t>INEP3</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Alpargatas</t>
+          <t>Inepar</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>25500</v>
+        <v>25400</v>
       </c>
       <c r="D246" t="n">
-        <v>4706682368</v>
+        <v>65073812</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>INEP3</t>
+          <t>ENGI4</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Inepar</t>
+          <t>Energisa</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>25400</v>
+        <v>24400</v>
       </c>
       <c r="D247" t="n">
-        <v>65073812</v>
+        <v>20799023104</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>ENGI4</t>
+          <t>ALLD3</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Energisa</t>
+          <t>Allied</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>24400</v>
+        <v>23200</v>
       </c>
       <c r="D248" t="n">
-        <v>20799023104</v>
+        <v>663115968</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>ALLD3</t>
+          <t>KRSA3</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Allied</t>
+          <t>Kora Saúde</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>23200</v>
+        <v>20700</v>
       </c>
       <c r="D249" t="n">
-        <v>663115968</v>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" s="1" t="inlineStr">
-        <is>
-          <t>KRSA3</t>
-        </is>
-      </c>
-      <c r="B250" t="inlineStr">
-        <is>
-          <t>Kora Saúde</t>
-        </is>
-      </c>
-      <c r="C250" t="n">
-        <v>20700</v>
-      </c>
-      <c r="D250" t="n">
         <v>674443776</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajustando função de detectar_martelos.py, pois após alteração anterior, havia quebrado
</commit_message>
<xml_diff>
--- a/Bases/Lista de ações Tratada.xlsx
+++ b/Bases/Lista de ações Tratada.xlsx
@@ -8234,7 +8234,7 @@
         <v>0.16244721</v>
       </c>
       <c r="AE33">
-        <v>0.202009</v>
+        <v>0.235195</v>
       </c>
       <c r="AF33">
         <v>1745539200</v>
@@ -11897,10 +11897,10 @@
         <v>-0.35174745</v>
       </c>
       <c r="AE54">
-        <v>0.25</v>
+        <v>0.450164</v>
       </c>
       <c r="AF54">
-        <v>1723766400</v>
+        <v>1741305600</v>
       </c>
       <c r="AG54">
         <v>2.6875</v>
@@ -15560,7 +15560,7 @@
         <v>0.08237707599999999</v>
       </c>
       <c r="AE75">
-        <v>0.074072</v>
+        <v>0.074027</v>
       </c>
       <c r="AF75">
         <v>1744588800</v>
@@ -18609,10 +18609,10 @@
         <v>0.20395005</v>
       </c>
       <c r="AE92">
-        <v>0.156105</v>
+        <v>0.202583</v>
       </c>
       <c r="AF92">
-        <v>1727395200</v>
+        <v>1734566400</v>
       </c>
       <c r="AG92">
         <v>1.58333</v>
@@ -21831,10 +21831,10 @@
         <v>-0.11806595</v>
       </c>
       <c r="AE110">
-        <v>1.39228</v>
+        <v>0.153465</v>
       </c>
       <c r="AF110">
-        <v>1735776000</v>
+        <v>1717113600</v>
       </c>
       <c r="AG110">
         <v>2.66667</v>
@@ -22189,10 +22189,10 @@
         <v>0.09348202</v>
       </c>
       <c r="AE112">
-        <v>0.783358</v>
+        <v>1.610052</v>
       </c>
       <c r="AF112">
-        <v>1692316800</v>
+        <v>1745971200</v>
       </c>
       <c r="AG112">
         <v>2.72727</v>
@@ -23946,10 +23946,10 @@
         <v>0.37148666</v>
       </c>
       <c r="AE122">
-        <v>0.605805</v>
+        <v>0.421051</v>
       </c>
       <c r="AF122">
-        <v>1743379200</v>
+        <v>1735776000</v>
       </c>
       <c r="AG122">
         <v>1.63636</v>
@@ -24838,10 +24838,10 @@
         <v>-0.2983871</v>
       </c>
       <c r="AE127">
-        <v>0.274569</v>
+        <v>0.185884</v>
       </c>
       <c r="AF127">
-        <v>1741219200</v>
+        <v>1722556800</v>
       </c>
       <c r="AG127">
         <v>1.88889</v>
@@ -25202,7 +25202,7 @@
         <v>-0.24482208</v>
       </c>
       <c r="AE129">
-        <v>0.324923</v>
+        <v>0.093081</v>
       </c>
       <c r="AF129">
         <v>1744329600</v>
@@ -42963,10 +42963,10 @@
         <v>-0.6054945</v>
       </c>
       <c r="AE233">
-        <v>47.55625</v>
+        <v>510.689</v>
       </c>
       <c r="AF233">
-        <v>1207699200</v>
+        <v>1363910400</v>
       </c>
       <c r="AH233" t="s">
         <v>683</v>
@@ -45184,10 +45184,10 @@
         <v>-0.12364131</v>
       </c>
       <c r="AE247">
-        <v>0.212294</v>
+        <v>0.270746</v>
       </c>
       <c r="AF247">
-        <v>1699315200</v>
+        <v>1730246400</v>
       </c>
       <c r="AH247" t="s">
         <v>683</v>
@@ -45354,7 +45354,7 @@
         <v>0.08</v>
       </c>
       <c r="AF248">
-        <v>1744848000</v>
+        <v>1731888000</v>
       </c>
       <c r="AH248" t="s">
         <v>683</v>

</xml_diff>

<commit_message>
Criação da função que apenas gera o histórico, gerar_arquivo_historico, sem processar a base de análise
</commit_message>
<xml_diff>
--- a/Bases/Lista de ações Tratada.xlsx
+++ b/Bases/Lista de ações Tratada.xlsx
@@ -13341,7 +13341,7 @@
         <v>0.2260766</v>
       </c>
       <c r="AF60">
-        <v>0.213813</v>
+        <v>0.183644</v>
       </c>
       <c r="AG60">
         <v>1745539200</v>
@@ -30214,10 +30214,10 @@
         <v>0.3409648</v>
       </c>
       <c r="AF155">
-        <v>0.596564</v>
+        <v>0.65</v>
       </c>
       <c r="AG155">
-        <v>1747872000</v>
+        <v>1731456000</v>
       </c>
       <c r="AH155">
         <v>1.2</v>
@@ -33928,7 +33928,7 @@
         <v>0.5</v>
       </c>
       <c r="AF176">
-        <v>0.3</v>
+        <v>0.300639</v>
       </c>
       <c r="AG176">
         <v>1745798400</v>

</xml_diff>

<commit_message>
Ajustada também a função de detectar_martelos_todos_os_tickers para gerar o arquivo de Histórico corretamente
</commit_message>
<xml_diff>
--- a/Bases/Lista de ações Tratada.xlsx
+++ b/Bases/Lista de ações Tratada.xlsx
@@ -13341,7 +13341,7 @@
         <v>0.2260766</v>
       </c>
       <c r="AF60">
-        <v>0.183644</v>
+        <v>0.213813</v>
       </c>
       <c r="AG60">
         <v>1745539200</v>
@@ -23647,7 +23647,7 @@
         <v>-0.21875</v>
       </c>
       <c r="AF119">
-        <v>0.093081</v>
+        <v>0.324923</v>
       </c>
       <c r="AG119">
         <v>1744329600</v>
@@ -33561,7 +33561,7 @@
         <v>0.73131776</v>
       </c>
       <c r="AF174">
-        <v>0.204417</v>
+        <v>0.8221580000000001</v>
       </c>
       <c r="AG174">
         <v>1746144000</v>
@@ -33928,7 +33928,7 @@
         <v>0.5</v>
       </c>
       <c r="AF176">
-        <v>0.300639</v>
+        <v>0.3</v>
       </c>
       <c r="AG176">
         <v>1745798400</v>

</xml_diff>